<commit_message>
added all trade studies to power point
</commit_message>
<xml_diff>
--- a/Fall 2025/Aero Design 1/Trade Studies/Antenna Trade Study.xlsx
+++ b/Fall 2025/Aero Design 1/Trade Studies/Antenna Trade Study.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noaht\School\Fall 2025\Aero Design 1\Trade Studies\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noahtouchton/School_Git/School/Fall 2025/Aero Design 1/Trade Studies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C1DCBC8-6990-4A2C-A0F1-834E23EA90DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA742AB-069A-674C-9E8E-73516F17838D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CBE0DF9F-DDFE-4833-8F35-1B1A204C32DC}"/>
+    <workbookView xWindow="4420" yWindow="800" windowWidth="27160" windowHeight="20960" xr2:uid="{CBE0DF9F-DDFE-4833-8F35-1B1A204C32DC}"/>
   </bookViews>
   <sheets>
     <sheet name="TS" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>Part:</t>
   </si>
@@ -223,13 +223,13 @@
     <t>Avaliability/Cost</t>
   </si>
   <si>
-    <t>ISIS S-Band Patch</t>
-  </si>
-  <si>
     <t>EnduroSat Patch</t>
   </si>
   <si>
     <t>Anywaves Patch</t>
+  </si>
+  <si>
+    <t>ISISPACE S-Band Patch</t>
   </si>
 </sst>
 </file>
@@ -294,7 +294,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -682,12 +682,56 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -762,39 +806,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -816,6 +827,39 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -832,6 +876,30 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1188,98 +1256,96 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC4302AA-4CFD-4C9C-A5EA-EC60A679F4CF}">
   <dimension ref="A1:N17"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="5" width="14.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
-    <col min="7" max="8" width="10.140625" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="4.33203125" customWidth="1"/>
+    <col min="4" max="5" width="14.5" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="8" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="40"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C1" s="29"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="42"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C2" s="31"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="42"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C3" s="31"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="43">
+      <c r="B4" s="32">
         <v>45916</v>
       </c>
-      <c r="C4" s="44"/>
-    </row>
-    <row r="5" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="45" t="s">
+      <c r="C4" s="33"/>
+    </row>
+    <row r="5" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="34"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
     </row>
-    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="31" t="s">
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="40"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="32"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="28" t="s">
+      <c r="J9" s="37"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="J9" s="29"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="M9" s="32"/>
-      <c r="N9" s="33"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
+      <c r="M9" s="40"/>
+      <c r="N9" s="41"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B10" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="16" t="s">
-        <v>7</v>
-      </c>
+      <c r="C10" s="53"/>
       <c r="D10" s="16" t="s">
         <v>6</v>
       </c>
@@ -1314,11 +1380,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B11" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="22"/>
+      <c r="C11" s="55"/>
       <c r="D11" s="23">
         <v>25</v>
       </c>
@@ -1359,11 +1425,11 @@
         <v>7.6923076923076925</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="5" t="s">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="24"/>
+      <c r="C12" s="57"/>
       <c r="D12" s="23">
         <v>20</v>
       </c>
@@ -1404,11 +1470,11 @@
         <v>6.6666666666666661</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B13" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="24"/>
+      <c r="C13" s="57"/>
       <c r="D13" s="23">
         <v>20</v>
       </c>
@@ -1449,11 +1515,11 @@
         <v>6.1538461538461542</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="5" t="s">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B14" s="56" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="24"/>
+      <c r="C14" s="57"/>
       <c r="D14" s="23">
         <v>15</v>
       </c>
@@ -1494,11 +1560,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="5" t="s">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B15" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="24"/>
+      <c r="C15" s="57"/>
       <c r="D15" s="23">
         <v>10</v>
       </c>
@@ -1539,11 +1605,11 @@
         <v>3.333333333333333</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="5" t="s">
+    <row r="16" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="24"/>
+      <c r="C16" s="59"/>
       <c r="D16" s="23">
         <v>10</v>
       </c>
@@ -1584,13 +1650,13 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="2:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="36" t="s">
+    <row r="17" spans="2:14" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="38"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="45"/>
       <c r="F17" s="13"/>
       <c r="G17" s="14"/>
       <c r="H17" s="27">
@@ -1611,17 +1677,24 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="17">
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="B17:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1630,54 +1703,54 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C407BE7C-5C9C-4832-909A-18821EF79075}">
   <dimension ref="A1:K22"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12" s="21" t="s">
         <v>31</v>
       </c>
@@ -1690,7 +1763,7 @@
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B13" s="21" t="s">
         <v>32</v>
       </c>
@@ -1703,7 +1776,7 @@
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B14" s="21" t="s">
         <v>33</v>
       </c>
@@ -1716,8 +1789,8 @@
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B16" s="46" t="s">
         <v>17</v>
       </c>
@@ -1729,13 +1802,13 @@
       </c>
       <c r="G16" s="50"/>
       <c r="H16" s="51"/>
-      <c r="I16" s="28" t="s">
+      <c r="I16" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="J16" s="29"/>
-      <c r="K16" s="30"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J16" s="37"/>
+      <c r="K16" s="38"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B17" s="8" t="s">
         <v>4</v>
       </c>
@@ -1767,7 +1840,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B18" s="9" t="s">
         <v>29</v>
       </c>
@@ -1803,7 +1876,7 @@
         <v>0.74702380952380965</v>
       </c>
     </row>
-    <row r="19" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
         <v>30</v>
       </c>
@@ -1839,13 +1912,13 @@
         <v>0.15625</v>
       </c>
     </row>
-    <row r="20" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="36" t="s">
+    <row r="20" spans="2:11" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="45"/>
       <c r="F20" s="13"/>
       <c r="G20" s="14"/>
       <c r="H20" s="27">
@@ -1859,7 +1932,7 @@
         <v>0.90327380952380965</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B22" s="21" t="s">
         <v>34</v>
       </c>
@@ -1876,6 +1949,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="619bfd31-fbc9-4e3d-b639-5680fd0427c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100445E206EC97B5241AE364FC742D190F1" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8284591227d7a4ff90c48262bf6356f1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="619bfd31-fbc9-4e3d-b639-5680fd0427c3" xmlns:ns3="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b29a3fb53242aaf6387bf4e700398a19" ns2:_="" ns3:_="">
     <xsd:import namespace="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
@@ -2130,41 +2223,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="619bfd31-fbc9-4e3d-b639-5680fd0427c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F6E05F-13AA-425A-905B-6BF8E82F9AC9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1748E98C-71FF-4E5A-BAD7-3F9220D62AE3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
-    <ds:schemaRef ds:uri="37bd234a-b872-4d8f-a05f-9ce9a06b0a24"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2187,9 +2249,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1748E98C-71FF-4E5A-BAD7-3F9220D62AE3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F6E05F-13AA-425A-905B-6BF8E82F9AC9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
+    <ds:schemaRef ds:uri="37bd234a-b872-4d8f-a05f-9ce9a06b0a24"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>